<commit_message>
feat(backend): implement search APIs
</commit_message>
<xml_diff>
--- a/docs/specs/snaphere-api-spec-v1.1.5.xlsx
+++ b/docs/specs/snaphere-api-spec-v1.1.5.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0. 개요" sheetId="1" r:id="R12d827777b0e44fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. API 목록" sheetId="2" r:id="R96b920b6f27c4cee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. 요청 파라미터" sheetId="3" r:id="Rd711201cf950424d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. 응답 스키마" sheetId="4" r:id="Rf093336020bc45d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. 공통 규약" sheetId="5" r:id="Re7bbe8a0e5454d46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. 에러 코드" sheetId="6" r:id="R039f7824e0284737"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. 배치·비동기" sheetId="7" r:id="R0e2491da54264f9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. 요구사항 추적" sheetId="8" r:id="R7a59adfc22c047f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. ERD 엔터티" sheetId="9" r:id="Rca2e6fc396dc499e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. ERD 관계" sheetId="10" r:id="R2e2ffc762c1d438f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0. 개요" sheetId="1" r:id="R5884414492c249d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. API 목록" sheetId="2" r:id="R277d73defaba4cc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. 요청 파라미터" sheetId="3" r:id="R5855b853d5284058"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. 응답 스키마" sheetId="4" r:id="R6dfb7574134f4606"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. 공통 규약" sheetId="5" r:id="Re1400ff3c95d4c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. 에러 코드" sheetId="6" r:id="R8f8e03bd7edc480e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. 배치·비동기" sheetId="7" r:id="R4209a4ace7704e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. 요구사항 추적" sheetId="8" r:id="R066a3b605ada4ef7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. ERD 엔터티" sheetId="9" r:id="R72ad145913764f36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. ERD 관계" sheetId="10" r:id="Ra8258899434b4058"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -145,7 +145,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="54">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -272,6 +272,15 @@
           <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
         </x:ext>
       </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1870,21 +1879,17 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="60">
+    <x:row r="60" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A60" s="40" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">D-9</x:t>
         </x:is>
       </x:c>
-      <x:c r="B60" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">남은 미결</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C60" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">최근 검색어(SCH-011)·최근 본 장소(VST-006) 저장소는 DBML 미결정 10 — API 비고에 그대로 표기</x:t>
-        </x:is>
+      <x:c r="B60" s="51" t="str">
+        <x:v>검색 저장소</x:v>
+      </x:c>
+      <x:c r="C60" s="51" t="str">
+        <x:v>최근 검색어(SCH-011)는 Redis에 사용자별 최대 20개·TTL 30일로 저장. 최근 본 장소(VST-006)는 별도 결정 유지</x:v>
       </x:c>
       <x:c r="D60" s="40" t="inlineStr">
         <x:is>
@@ -3184,7 +3189,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc654fc8c17bf45a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a346d53762144f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9868,7 +9873,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="85" s="33" customFormat="1" ht="64.80000305175781" customHeight="1">
+    <x:row r="85" s="33" customFormat="1" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A85" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">API-SCH-001</x:t>
@@ -9904,53 +9909,49 @@
           <x:t xml:space="preserve">Must</x:t>
         </x:is>
       </x:c>
-      <x:c r="H85" s="37" t="inlineStr">
+      <x:c r="H85" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">장소·게시글·사용자·태그를 통합 검색하고 타입별 상위를 반환한다.</x:t>
         </x:is>
       </x:c>
-      <x:c r="I85" s="37" t="inlineStr">
+      <x:c r="I85" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
-      <x:c r="J85" s="37" t="inlineStr">
+      <x:c r="J85" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SearchResult</x:t>
         </x:is>
       </x:c>
-      <x:c r="K85" s="37" t="inlineStr">
+      <x:c r="K85" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">200</x:t>
         </x:is>
       </x:c>
-      <x:c r="L85" s="37" t="inlineStr">
+      <x:c r="L85" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">COMMON_400, AUTH_REQUIRED, COMMON_500</x:t>
         </x:is>
       </x:c>
-      <x:c r="M85" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">타입별 cursor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N85" s="37" t="inlineStr">
+      <x:c r="M85" s="52" t="str">
+        <x:v>단일 types 지정 시 불투명 keyset cursor</x:v>
+      </x:c>
+      <x:c r="N85" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
-      <x:c r="O85" s="37" t="inlineStr">
+      <x:c r="O85" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SCH-001, SCH-003~009</x:t>
         </x:is>
       </x:c>
-      <x:c r="P85" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">places, posts, users, tags, search_logs</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="86" s="33" customFormat="1" ht="64.80000305175781" customHeight="1">
+      <x:c r="P85" s="52" t="str">
+        <x:v>places, posts, users, tags, search_logs(커서 없는 첫 페이지 검색만 기록)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A86" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">API-SCH-002</x:t>
@@ -9986,53 +9987,49 @@
           <x:t xml:space="preserve">Could</x:t>
         </x:is>
       </x:c>
-      <x:c r="H86" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">검색 로그 집계 기반 인기 검색어를 반환한다.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I86" s="37" t="inlineStr">
+      <x:c r="H86" s="52" t="str">
+        <x:v>최근 7일 검색 로그 집계 기반 인기 검색어를 반환한다.</x:v>
+      </x:c>
+      <x:c r="I86" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
-      <x:c r="J86" s="37" t="inlineStr">
+      <x:c r="J86" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">PopularKeyword[]</x:t>
         </x:is>
       </x:c>
-      <x:c r="K86" s="37" t="inlineStr">
+      <x:c r="K86" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">200</x:t>
         </x:is>
       </x:c>
-      <x:c r="L86" s="37" t="inlineStr">
+      <x:c r="L86" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">COMMON_400, AUTH_REQUIRED, COMMON_500</x:t>
         </x:is>
       </x:c>
-      <x:c r="M86" s="37" t="inlineStr">
+      <x:c r="M86" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
-      <x:c r="N86" s="37" t="inlineStr">
+      <x:c r="N86" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">10m</x:t>
         </x:is>
       </x:c>
-      <x:c r="O86" s="37" t="inlineStr">
+      <x:c r="O86" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SCH-002, SCH-010</x:t>
         </x:is>
       </x:c>
-      <x:c r="P86" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">search_logs</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="87" s="33" customFormat="1" ht="64.80000305175781" customHeight="1">
+      <x:c r="P86" s="52" t="str">
+        <x:v>search_logs(30일 보존), Redis(10분 캐시)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A87" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">API-SCH-003</x:t>
@@ -10068,53 +10065,51 @@
           <x:t xml:space="preserve">Could</x:t>
         </x:is>
       </x:c>
-      <x:c r="H87" s="37" t="inlineStr">
+      <x:c r="H87" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">사용자의 최근 검색어를 조회한다.</x:t>
         </x:is>
       </x:c>
-      <x:c r="I87" s="37" t="inlineStr">
+      <x:c r="I87" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
-      <x:c r="J87" s="37" t="inlineStr">
+      <x:c r="J87" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">RecentSearch[]</x:t>
         </x:is>
       </x:c>
-      <x:c r="K87" s="37" t="inlineStr">
+      <x:c r="K87" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">200</x:t>
         </x:is>
       </x:c>
-      <x:c r="L87" s="37" t="inlineStr">
+      <x:c r="L87" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">COMMON_400, AUTH_REQUIRED, COMMON_500</x:t>
         </x:is>
       </x:c>
-      <x:c r="M87" s="37" t="inlineStr">
+      <x:c r="M87" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
-      <x:c r="N87" s="37" t="inlineStr">
+      <x:c r="N87" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
-      <x:c r="O87" s="37" t="inlineStr">
+      <x:c r="O87" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SCH-002, SCH-011</x:t>
         </x:is>
       </x:c>
-      <x:c r="P87" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">search_logs / ※ 최근 검색어 저장소 미정 — 앱 로컬·Redis·별도 테이블 (DBML 미결정 10)</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="88" s="33" customFormat="1" ht="118.80000305175781" customHeight="1">
+      <x:c r="P87" s="52" t="str">
+        <x:v>Redis(사용자별 최대 20개, TTL 30일, 동일 검색어 최신화)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A88" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">API-SCH-004</x:t>
@@ -10150,50 +10145,48 @@
           <x:t xml:space="preserve">Could</x:t>
         </x:is>
       </x:c>
-      <x:c r="H88" s="37" t="inlineStr">
+      <x:c r="H88" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">최근 검색어 한 건 또는 전체를 삭제한다.</x:t>
         </x:is>
       </x:c>
-      <x:c r="I88" s="37" t="inlineStr">
+      <x:c r="I88" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
-      <x:c r="J88" s="37" t="inlineStr">
+      <x:c r="J88" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Empty</x:t>
         </x:is>
       </x:c>
-      <x:c r="K88" s="37" t="inlineStr">
+      <x:c r="K88" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">204</x:t>
         </x:is>
       </x:c>
-      <x:c r="L88" s="37" t="inlineStr">
+      <x:c r="L88" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">COMMON_400, AUTH_REQUIRED, COMMON_500</x:t>
         </x:is>
       </x:c>
-      <x:c r="M88" s="37" t="inlineStr">
+      <x:c r="M88" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
-      <x:c r="N88" s="37" t="inlineStr">
+      <x:c r="N88" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
-      <x:c r="O88" s="37" t="inlineStr">
+      <x:c r="O88" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SCH-011</x:t>
         </x:is>
       </x:c>
-      <x:c r="P88" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">search_logs</x:t>
-        </x:is>
+      <x:c r="P88" s="52" t="str">
+        <x:v>Redis(검색어 1건 또는 전체 삭제)</x:v>
       </x:c>
     </x:row>
     <x:row r="89" s="33" customFormat="1" ht="64.80000305175781" customHeight="1">
@@ -11283,7 +11276,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67f956d6004945ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc40bba46128a4a00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21198,7 +21191,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="198" s="33" customFormat="1" ht="21.600000381469727" customHeight="1">
+    <x:row r="198" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A198" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">API-SCH-001</x:t>
@@ -21234,10 +21227,8 @@
           <x:t xml:space="preserve">N</x:t>
         </x:is>
       </x:c>
-      <x:c r="H198" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PLACE|POST|USER|TAG</x:t>
-        </x:is>
+      <x:c r="H198" s="52" t="str">
+        <x:v>PLACE|POST|USER|TAG, cursor 사용 시 정확히 1개</x:v>
       </x:c>
       <x:c r="I198" s="37" t="inlineStr">
         <x:is>
@@ -21250,7 +21241,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="199" s="33" customFormat="1" ht="32.400001525878906" customHeight="1">
+    <x:row r="199" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A199" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">API-SCH-001</x:t>
@@ -21286,10 +21277,8 @@
           <x:t xml:space="preserve">N</x:t>
         </x:is>
       </x:c>
-      <x:c r="H199" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">필터</x:t>
-        </x:is>
+      <x:c r="H199" s="52" t="str">
+        <x:v>지역명과 정확히 일치하면 해당 지역 코드가 우선</x:v>
       </x:c>
       <x:c r="I199" s="37" t="inlineStr">
         <x:is>
@@ -21302,7 +21291,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="200" s="33" customFormat="1" ht="32.400001525878906" customHeight="1">
+    <x:row r="200" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A200" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">API-SCH-001</x:t>
@@ -21338,10 +21327,8 @@
           <x:t xml:space="preserve">N</x:t>
         </x:is>
       </x:c>
-      <x:c r="H200" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">더보기 타입의 커서</x:t>
-        </x:is>
+      <x:c r="H200" s="52" t="str">
+        <x:v>단일 검색 타입용 불투명 keyset cursor</x:v>
       </x:c>
       <x:c r="I200" s="37" t="inlineStr">
         <x:is>
@@ -21354,7 +21341,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="201" s="33" customFormat="1" ht="32.400001525878906" customHeight="1">
+    <x:row r="201" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A201" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">API-SCH-001</x:t>
@@ -21390,7 +21377,7 @@
           <x:t xml:space="preserve">N</x:t>
         </x:is>
       </x:c>
-      <x:c r="H201" s="37" t="inlineStr">
+      <x:c r="H201" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">타입별 기본 5, 더보기 최대 50</x:t>
         </x:is>
@@ -21404,7 +21391,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="202" s="33" customFormat="1" ht="32.400001525878906" customHeight="1">
+    <x:row r="202" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A202" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">API-SCH-002</x:t>
@@ -21440,7 +21427,7 @@
           <x:t xml:space="preserve">N</x:t>
         </x:is>
       </x:c>
-      <x:c r="H202" s="37" t="inlineStr">
+      <x:c r="H202" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">-</x:t>
         </x:is>
@@ -21456,7 +21443,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="203" s="33" customFormat="1" ht="32.400001525878906" customHeight="1">
+    <x:row r="203" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A203" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">API-SCH-002</x:t>
@@ -21492,10 +21479,8 @@
           <x:t xml:space="preserve">N</x:t>
         </x:is>
       </x:c>
-      <x:c r="H203" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">기본 10</x:t>
-        </x:is>
+      <x:c r="H203" s="52" t="str">
+        <x:v>기본 10, 최대 50</x:v>
       </x:c>
       <x:c r="I203" s="37" t="n">
         <x:v>10</x:v>
@@ -23374,7 +23359,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47ec598875e54713"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43dc20b6cebc4012"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33995,7 +33980,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="297" s="33" customFormat="1" ht="21.600000381469727" customHeight="1">
+    <x:row r="297" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A297" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">RecentSearch</x:t>
@@ -34021,18 +34006,14 @@
           <x:t xml:space="preserve">검색 로그 ID</x:t>
         </x:is>
       </x:c>
-      <x:c r="F297" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">sch_01</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G297" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">search_logs</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="298" s="33" customFormat="1" ht="21.600000381469727" customHeight="1">
+      <x:c r="F297" s="52" t="str">
+        <x:v>550e8400-e29b-41d4-a716-446655440000</x:v>
+      </x:c>
+      <x:c r="G297" s="52" t="str">
+        <x:v>Redis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="298" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A298" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">RecentSearch</x:t>
@@ -34058,18 +34039,16 @@
           <x:t xml:space="preserve">검색어</x:t>
         </x:is>
       </x:c>
-      <x:c r="F298" s="37" t="inlineStr">
+      <x:c r="F298" s="52" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">경복궁</x:t>
         </x:is>
       </x:c>
-      <x:c r="G298" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">search_logs</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="299" s="33" customFormat="1" ht="21.600000381469727" customHeight="1">
+      <x:c r="G298" s="52" t="str">
+        <x:v>Redis</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="299" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A299" s="45" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">RecentSearch</x:t>
@@ -34095,15 +34074,13 @@
           <x:t xml:space="preserve">검색 시각</x:t>
         </x:is>
       </x:c>
-      <x:c r="F299" s="46" t="inlineStr">
+      <x:c r="F299" s="53" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">예: 2026-09-01T09:00:00+09:00</x:t>
         </x:is>
       </x:c>
-      <x:c r="G299" s="46" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">search_logs</x:t>
-        </x:is>
+      <x:c r="G299" s="53" t="str">
+        <x:v>Redis</x:v>
       </x:c>
     </x:row>
     <x:row r="300" s="33" customFormat="1" ht="21.600000381469727" customHeight="1">
@@ -35259,7 +35236,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb159703a09a24102"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb480bbbd2ff4f38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35915,7 +35892,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf4037cd02f74f3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9bb24f5de324496"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37621,7 +37598,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43e4e96357354eef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1b80956fc6d4a40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38249,7 +38226,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba54ab3ab10e45c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e2f3f81516b47bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -50162,7 +50139,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="273" s="33" customFormat="1" ht="32.400001525878906" customHeight="1">
+    <x:row r="273" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A273" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SCH-010</x:t>
@@ -50199,13 +50176,11 @@
         </x:is>
       </x:c>
       <x:c r="H273" s="37" t="str"/>
-      <x:c r="I273" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">엔드포인트 계약에 직접 반영</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="274" s="33" customFormat="1" ht="43.20000076293945" customHeight="1">
+      <x:c r="I273" s="52" t="str">
+        <x:v>최근 7일 검색 로그 집계, Redis 10분 캐시, 로그 30일 보존</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="274" s="33" customFormat="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A274" s="37" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SCH-011</x:t>
@@ -50242,10 +50217,8 @@
         </x:is>
       </x:c>
       <x:c r="H274" s="37" t="str"/>
-      <x:c r="I274" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">엔드포인트 계약에 직접 반영</x:t>
-        </x:is>
+      <x:c r="I274" s="52" t="str">
+        <x:v>Redis 사용자별 최대 20개, TTL 30일; 동일 검색어는 최신 순서로 갱신</x:v>
       </x:c>
     </x:row>
     <x:row r="275" s="33" customFormat="1" ht="54" customHeight="1">
@@ -51221,7 +51194,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R646cc4da6ffe4c8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cf7e94829a64c34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52067,7 +52040,7 @@
         <x:v>조합 단위 동기화 결과 기록</x:v>
       </x:c>
     </x:row>
-    <x:row r="32">
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="37" t="str">
         <x:v>운영</x:v>
       </x:c>
@@ -52092,8 +52065,8 @@
       <x:c r="H32" s="37" t="str">
         <x:v>SCH-010</x:v>
       </x:c>
-      <x:c r="I32" s="37" t="str">
-        <x:v>인기 검색어 집계용. user_id 없음</x:v>
+      <x:c r="I32" s="52" t="str">
+        <x:v>인기 검색어 집계용. user_id 없음. 최근 7일 집계·30일 보존</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -52114,7 +52087,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f01753ff2354924"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R883619f92ba443bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>